<commit_message>
ice exchange pre and post
</commit_message>
<xml_diff>
--- a/MORITZ APA 136.xlsx
+++ b/MORITZ APA 136.xlsx
@@ -8,36 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/moriheidtmann/Documents/Work/Playwrite_VS_Extention/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9F69131-C58E-594C-A453-4C81EAD3FC11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF3ECAC7-2C29-0540-B157-8FA115D4A959}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
-    <sheet name="SORTED" sheetId="2" r:id="rId2"/>
-    <sheet name="OVERWIEW" sheetId="15" r:id="rId3"/>
-    <sheet name="GREECE" sheetId="13" r:id="rId4"/>
-    <sheet name="HUNGARY" sheetId="11" r:id="rId5"/>
-    <sheet name="Nordic" sheetId="10" r:id="rId6"/>
-    <sheet name="BALTIC" sheetId="12" r:id="rId7"/>
-    <sheet name="CZECH REPUBLIC" sheetId="9" r:id="rId8"/>
-    <sheet name="NETHERLANDS" sheetId="6" r:id="rId9"/>
-    <sheet name="FRANCE" sheetId="5" r:id="rId10"/>
-    <sheet name="GERMANY" sheetId="3" r:id="rId11"/>
-    <sheet name="ITALY" sheetId="4" r:id="rId12"/>
-    <sheet name="BULGARIA" sheetId="8" r:id="rId13"/>
-    <sheet name="INFO" sheetId="7" r:id="rId14"/>
+    <sheet name="OVERWIEW" sheetId="15" r:id="rId1"/>
+    <sheet name="Worksheet" sheetId="1" r:id="rId2"/>
+    <sheet name="SORTED" sheetId="2" r:id="rId3"/>
+    <sheet name="GERMANY" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">GERMANY!$A$1:$A$1048461</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">SORTED!$D$1:$D$140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">GERMANY!$A$1:$A$1048461</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">SORTED!$D$1:$D$140</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3861" uniqueCount="1077">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3632" uniqueCount="1069">
   <si>
     <t>ae_authorisationNotificationDateStr</t>
   </si>
@@ -3096,15 +3086,6 @@
     <t>Deutsche Börse AG manages the relationship with the client with respect to MiFIR Data Products for the Deutsche Börse Group trading venues, such as EEX, Eurex, and XETRA simplifying access. </t>
   </si>
   <si>
-    <t>https://www.ice.com/futures-europe/mifidii</t>
-  </si>
-  <si>
-    <t>commodities</t>
-  </si>
-  <si>
-    <t>infrastructure</t>
-  </si>
-  <si>
     <t>EURONEXT</t>
   </si>
   <si>
@@ -3114,30 +3095,6 @@
     <t>https://www.bse-sofia.bg/en/apa-trading-data</t>
   </si>
   <si>
-    <t>DONE</t>
-  </si>
-  <si>
-    <t>https://prices.wienerborse.at/#tab-content1</t>
-  </si>
-  <si>
-    <t>LUXEMBURG</t>
-  </si>
-  <si>
-    <t>https://www.athexgroup.gr/en/market-data/data-services/delayed-feed#:~:text=Pre,Access%20the%20related%20files%20here</t>
-  </si>
-  <si>
-    <t>Daten über XATH/XADE</t>
-  </si>
-  <si>
-    <t>https://www.enexgroup.gr/post-trade#:~:text=Post%20Trade%20Transparency%20for%20HENEX,midnight%20of%20the%20next%20business%C2%A0day</t>
-  </si>
-  <si>
-    <t>Daten über HENEX-Portal</t>
-  </si>
-  <si>
-    <t>https://www.bankofgreece.gr/en/main-tasks/markets/hdat/pre-trade-data#:~:text=HDAT%20makes%20pre,600%2F2014%20%28MIFIR</t>
-  </si>
-  <si>
     <t>NASDAQ</t>
   </si>
   <si>
@@ -3180,15 +3137,6 @@
     <t>https://www.mds.deutsche-boerse.com/mds-en/real-time-data/mifid-ii-disaggregated-information-products</t>
   </si>
   <si>
-    <t>alternative</t>
-  </si>
-  <si>
-    <t>https://www.bet.hu/site/Angol/pages/derivatives-market#:~:text=Magyar</t>
-  </si>
-  <si>
-    <t>https://bet.hu/site/Angol/Contents/Prices-and-Markets/Data-download#:~:text=Share%20section%3A%20Download</t>
-  </si>
-  <si>
     <t>Deutsche Börse Group</t>
   </si>
   <si>
@@ -3222,9 +3170,6 @@
     <t>NASDAQ Baltic</t>
   </si>
   <si>
-    <t>ICE is for startups i dont think they have a personal data vendor</t>
-  </si>
-  <si>
     <t>Bucharest</t>
   </si>
   <si>
@@ -3267,7 +3212,28 @@
     <t>https://www.borzamalta.com.mt/trading</t>
   </si>
   <si>
-    <t>CBOE &amp; Euronext&amp; ICE&amp; CME</t>
+    <t>ICE POST</t>
+  </si>
+  <si>
+    <t>https://www.ice.com/report/61</t>
+  </si>
+  <si>
+    <t>https://www.ice.com/report/60</t>
+  </si>
+  <si>
+    <t>CME</t>
+  </si>
+  <si>
+    <t>https://www.traxapa.com/apa-publication/#/trades</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CBOE &amp; Euronext </t>
+  </si>
+  <si>
+    <t>ICE PRE</t>
+  </si>
+  <si>
+    <t>NOT IN THE EU</t>
   </si>
 </sst>
 </file>
@@ -3335,7 +3301,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3366,14 +3332,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -3396,21 +3356,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -3426,7 +3371,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -3436,6 +3380,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -3740,6 +3685,368 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{916CD87E-FB8F-5F4E-9AB4-0BF93ECEEA89}">
+  <dimension ref="A1:F33"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="58.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="62.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>771</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1020</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>330</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="13" customFormat="1">
+      <c r="A3" s="13" t="s">
+        <v>676</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>1036</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>1055</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>319</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>1020</v>
+      </c>
+      <c r="F4" t="s">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="14" customFormat="1" ht="16">
+      <c r="A5" s="14" t="s">
+        <v>356</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>1058</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>1048</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>1057</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>1056</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>206</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>1020</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="13" customFormat="1">
+      <c r="A7" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="13" customFormat="1">
+      <c r="A8" s="13" t="s">
+        <v>382</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>1046</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="13" customFormat="1">
+      <c r="A9" s="13" t="s">
+        <v>239</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="13" customFormat="1">
+      <c r="A10" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="13" customFormat="1">
+      <c r="A11" s="13" t="s">
+        <v>250</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>1038</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="13" customFormat="1">
+      <c r="A12" s="13" t="s">
+        <v>607</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>1039</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>422</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>1053</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>1044</v>
+      </c>
+      <c r="E13" t="s">
+        <v>1054</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="13" customFormat="1">
+      <c r="A14" s="13" t="s">
+        <v>365</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
+        <v>665</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>181</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" s="13" customFormat="1">
+      <c r="A17" s="13" t="s">
+        <v>444</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>1046</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="13" customFormat="1">
+      <c r="A18" s="13" t="s">
+        <v>433</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>1046</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" s="12" customFormat="1" ht="20">
+      <c r="A19" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>1040</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>1040</v>
+      </c>
+      <c r="F19" s="16"/>
+    </row>
+    <row r="20" spans="1:6" s="13" customFormat="1" ht="20">
+      <c r="A20" s="13" t="s">
+        <v>404</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>1048</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>1060</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" s="13" customFormat="1">
+      <c r="A21" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" s="13" customFormat="1">
+      <c r="A22" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" s="13" customFormat="1">
+      <c r="A23" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" t="s">
+        <v>456</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>1041</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>1045</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>1050</v>
+      </c>
+      <c r="E24" t="s">
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" t="s">
+        <v>497</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" s="13" customFormat="1">
+      <c r="A26" s="13" t="s">
+        <v>865</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>1047</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" t="s">
+        <v>654</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>1043</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>1044</v>
+      </c>
+      <c r="E27" t="s">
+        <v>1049</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" t="s">
+        <v>345</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>1020</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" s="14" customFormat="1">
+      <c r="A29" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="B29" s="14" t="s">
+        <v>1042</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" s="13" customFormat="1">
+      <c r="A30" s="13" t="s">
+        <v>525</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>1061</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>1040</v>
+      </c>
+      <c r="D31" t="s">
+        <v>1062</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>1067</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>1040</v>
+      </c>
+      <c r="D32" s="18" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>1064</v>
+      </c>
+      <c r="D33" t="s">
+        <v>1065</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A1048467">
+    <sortCondition ref="A1:A1048467"/>
+  </sortState>
+  <hyperlinks>
+    <hyperlink ref="D32" r:id="rId1" xr:uid="{3D582A70-B0E5-A44F-89C8-C437C8ADF110}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AX140"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
@@ -13412,756 +13719,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41B1068A-70D8-5141-B56A-F887E4222AFE}">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" s="2" customFormat="1">
-      <c r="A1" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>1022</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>1021</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" s="2" customFormat="1">
-      <c r="A2" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>1022</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="2" customFormat="1">
-      <c r="A3" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>1022</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>1020</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" s="2" customFormat="1">
-      <c r="A4" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>1006</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>1022</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{190D282D-A498-5040-B7ED-BB0A4708E39A}">
-  <dimension ref="A1:F25"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="81.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="77.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="143.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="255.83203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>1013</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>1011</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" s="2" customFormat="1">
-      <c r="A2" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>1014</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="2" customFormat="1">
-      <c r="A3" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" s="2" customFormat="1">
-      <c r="A4" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="2" customFormat="1">
-      <c r="A5" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="2" customFormat="1">
-      <c r="A6" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="2" customFormat="1">
-      <c r="A7" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="2" customFormat="1">
-      <c r="A8" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="2" customFormat="1" ht="16" thickBot="1">
-      <c r="A9" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="2" customFormat="1" ht="16" thickBot="1">
-      <c r="A10" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>1010</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>1012</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" s="2" customFormat="1">
-      <c r="A11" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" s="4" customFormat="1">
-      <c r="A12" s="4" t="s">
-        <v>297</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>298</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>297</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" s="2" customFormat="1">
-      <c r="A13" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" s="2" customFormat="1">
-      <c r="A14" s="2" t="s">
-        <v>748</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>749</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>748</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>1018</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" s="2" customFormat="1">
-      <c r="A15" s="2" t="s">
-        <v>870</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>871</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>870</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>1017</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" s="2" customFormat="1">
-      <c r="A16" s="2" t="s">
-        <v>895</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>896</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>895</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>1015</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" s="2" customFormat="1">
-      <c r="A17" s="2" t="s">
-        <v>903</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>904</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>903</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>1015</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" s="4" customFormat="1">
-      <c r="A18" s="4" t="s">
-        <v>907</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>908</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>907</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" s="4" customFormat="1">
-      <c r="A19" s="4" t="s">
-        <v>911</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>912</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>911</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" s="2" customFormat="1">
-      <c r="A20" s="2" t="s">
-        <v>937</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>938</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>937</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" s="2" customFormat="1">
-      <c r="A21" s="2" t="s">
-        <v>946</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>947</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>946</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" s="2" customFormat="1">
-      <c r="A22" s="2" t="s">
-        <v>951</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>952</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>951</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>1016</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" s="2" customFormat="1">
-      <c r="A23" s="2" t="s">
-        <v>958</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>959</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>958</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>1016</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" s="2" customFormat="1">
-      <c r="A24" s="2" t="s">
-        <v>964</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>965</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>964</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>1016</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" s="2" customFormat="1">
-      <c r="A25" s="2" t="s">
-        <v>981</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>982</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>981</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>250</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:A1048461" xr:uid="{190D282D-A498-5040-B7ED-BB0A4708E39A}"/>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE3F7B10-E9D7-394E-88EE-E3C3786C779E}">
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="32.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" s="4" customFormat="1">
-      <c r="A2" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" s="4" customFormat="1">
-      <c r="A3" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" s="4" customFormat="1">
-      <c r="A4" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" s="2" customFormat="1">
-      <c r="A5" s="2" t="s">
-        <v>845</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>846</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>845</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" s="2" customFormat="1">
-      <c r="A6" s="2" t="s">
-        <v>852</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>853</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>852</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" s="4" customFormat="1">
-      <c r="A7" s="4" t="s">
-        <v>916</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>917</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>916</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>181</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C2F9903-2165-8846-946B-B401C9D8DB67}">
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="36.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="85.1640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="2" t="s">
-        <v>670</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>671</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>670</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>676</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>1024</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>1046</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>1047</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="2" t="s">
-        <v>681</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>682</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>681</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>676</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>1024</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="2" t="s">
-        <v>689</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>690</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>689</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>676</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>1024</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45DDC3CB-E423-7D48-9BE9-147CF6221632}">
-  <dimension ref="B5:C10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="5" spans="2:3">
-      <c r="B5" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>1022</v>
-      </c>
-    </row>
-    <row r="6" spans="2:3">
-      <c r="B6" s="1" t="s">
-        <v>330</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>1022</v>
-      </c>
-    </row>
-    <row r="7" spans="2:3">
-      <c r="B7" s="1" t="s">
-        <v>771</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>1023</v>
-      </c>
-    </row>
-    <row r="8" spans="2:3">
-      <c r="B8" s="1" t="s">
-        <v>319</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>1025</v>
-      </c>
-    </row>
-    <row r="9" spans="2:3">
-      <c r="B9" s="1" t="s">
-        <v>665</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>1022</v>
-      </c>
-    </row>
-    <row r="10" spans="2:3">
-      <c r="B10" s="1" t="s">
-        <v>1027</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD29CB13-D1F4-2448-8D40-3F8127B9D4DA}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:F140"/>
@@ -14203,7 +13761,7 @@
         <v>60</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>1033</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" hidden="1">
@@ -14234,7 +13792,7 @@
         <v>60</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>1039</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" hidden="1">
@@ -14269,7 +13827,7 @@
       <c r="A7" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="11" t="s">
         <v>95</v>
       </c>
       <c r="C7" s="3" t="s">
@@ -14293,7 +13851,7 @@
         <v>101</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>1042</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" hidden="1">
@@ -14310,7 +13868,7 @@
         <v>101</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>1043</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="10" spans="1:5" hidden="1">
@@ -14341,7 +13899,7 @@
         <v>101</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>1044</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="4" customFormat="1" hidden="1">
@@ -14358,7 +13916,7 @@
         <v>101</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>1044</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="2" customFormat="1" hidden="1">
@@ -14403,7 +13961,7 @@
         <v>101</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>1043</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="2" customFormat="1" hidden="1">
@@ -14420,7 +13978,7 @@
         <v>101</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>1043</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="2" customFormat="1" hidden="1">
@@ -14437,7 +13995,7 @@
         <v>101</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>1043</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="2" customFormat="1" hidden="1">
@@ -14454,7 +14012,7 @@
         <v>101</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>1043</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="19" spans="1:5" hidden="1">
@@ -14975,7 +14533,7 @@
         <v>456</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>1040</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="56" spans="1:5" s="2" customFormat="1" hidden="1">
@@ -14992,7 +14550,7 @@
         <v>456</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>1046</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="57" spans="1:5" s="2" customFormat="1" hidden="1">
@@ -15076,8 +14634,8 @@
       <c r="D61" s="4" t="s">
         <v>456</v>
       </c>
-      <c r="E61" s="11" t="s">
-        <v>1041</v>
+      <c r="E61" s="10" t="s">
+        <v>1030</v>
       </c>
     </row>
     <row r="62" spans="1:5" s="2" customFormat="1" hidden="1">
@@ -15125,7 +14683,7 @@
         <v>497</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>1045</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="65" spans="1:4" s="2" customFormat="1">
@@ -15484,7 +15042,7 @@
         <v>676</v>
       </c>
       <c r="E89" t="s">
-        <v>1024</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="90" spans="1:5" hidden="1">
@@ -15501,7 +15059,7 @@
         <v>676</v>
       </c>
       <c r="E90" t="s">
-        <v>1024</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="91" spans="1:5" hidden="1">
@@ -15518,7 +15076,7 @@
         <v>676</v>
       </c>
       <c r="E91" t="s">
-        <v>1024</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="92" spans="1:5" hidden="1">
@@ -15605,7 +15163,7 @@
         <v>101</v>
       </c>
       <c r="E97" s="4" t="s">
-        <v>1044</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="98" spans="1:6" hidden="1">
@@ -15692,10 +15250,10 @@
         <v>60</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>1034</v>
+        <v>1023</v>
       </c>
       <c r="F103" s="6" t="s">
-        <v>1035</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="104" spans="1:6" s="2" customFormat="1" hidden="1">
@@ -15711,11 +15269,11 @@
       <c r="D104" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E104" s="10" t="s">
-        <v>1034</v>
+      <c r="E104" s="9" t="s">
+        <v>1023</v>
       </c>
       <c r="F104" s="6" t="s">
-        <v>1035</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="105" spans="1:6" s="2" customFormat="1" hidden="1">
@@ -15732,10 +15290,10 @@
         <v>60</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>1034</v>
+        <v>1023</v>
       </c>
       <c r="F105" s="6" t="s">
-        <v>1035</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="106" spans="1:6" hidden="1">
@@ -15808,10 +15366,10 @@
         <v>60</v>
       </c>
       <c r="E110" s="6" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="F110" s="6" t="s">
-        <v>1036</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="111" spans="1:6" s="2" customFormat="1" hidden="1">
@@ -15828,10 +15386,10 @@
         <v>60</v>
       </c>
       <c r="E111" s="6" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="F111" s="6" t="s">
-        <v>1037</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="112" spans="1:6" s="2" customFormat="1" hidden="1">
@@ -15848,10 +15406,10 @@
         <v>60</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="F112" s="6" t="s">
-        <v>1038</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="113" spans="1:4" hidden="1">
@@ -16262,339 +15820,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{916CD87E-FB8F-5F4E-9AB4-0BF93ECEEA89}">
-  <dimension ref="A1:F30"/>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{190D282D-A498-5040-B7ED-BB0A4708E39A}">
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="58.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="62.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="81.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="77.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="143.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="255.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>771</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1023</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1058</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>330</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>1022</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="14" customFormat="1">
-      <c r="A3" s="14" t="s">
-        <v>676</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>1050</v>
-      </c>
-      <c r="F3" s="14" t="s">
-        <v>1070</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" t="s">
-        <v>319</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>1023</v>
-      </c>
-      <c r="F4" t="s">
-        <v>1067</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="15" customFormat="1" ht="16">
-      <c r="A5" s="15" t="s">
-        <v>356</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>1073</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>1063</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>1072</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>1071</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" t="s">
-        <v>206</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>1023</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>1058</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="14" customFormat="1">
-      <c r="A7" s="14" t="s">
-        <v>124</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>1051</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="14" customFormat="1">
-      <c r="A8" s="14" t="s">
-        <v>382</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>1060</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="14" customFormat="1">
-      <c r="A9" s="14" t="s">
-        <v>239</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>1051</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="14" customFormat="1">
-      <c r="A10" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>1022</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" s="14" customFormat="1">
-      <c r="A11" s="14" t="s">
-        <v>250</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>1052</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" s="14" customFormat="1">
-      <c r="A12" s="14" t="s">
-        <v>607</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>1053</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="A13" t="s">
-        <v>422</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>1068</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>1058</v>
-      </c>
-      <c r="E13" t="s">
-        <v>1069</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" s="14" customFormat="1">
-      <c r="A14" s="14" t="s">
-        <v>365</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>1051</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" t="s">
-        <v>665</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>1022</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" t="s">
-        <v>181</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>1022</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" s="14" customFormat="1">
-      <c r="A17" s="14" t="s">
-        <v>444</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>1060</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" s="14" customFormat="1">
-      <c r="A18" s="14" t="s">
-        <v>433</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>1060</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" s="13" customFormat="1" ht="20">
-      <c r="A19" s="13" t="s">
-        <v>227</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>1054</v>
-      </c>
-      <c r="C19" s="13" t="s">
-        <v>1054</v>
-      </c>
-      <c r="F19" s="17"/>
-    </row>
-    <row r="20" spans="1:6" s="14" customFormat="1" ht="20">
-      <c r="A20" s="14" t="s">
-        <v>404</v>
-      </c>
-      <c r="B20" s="14" t="s">
-        <v>1050</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>1063</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>1075</v>
-      </c>
-      <c r="F20" s="18" t="s">
-        <v>1074</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" t="s">
-        <v>393</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>1076</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>1061</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" s="14" customFormat="1">
-      <c r="A22" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>1051</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" s="14" customFormat="1">
-      <c r="A23" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>1051</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6">
-      <c r="A24" t="s">
-        <v>456</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>1055</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>1059</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>1065</v>
-      </c>
-      <c r="E24" t="s">
-        <v>1066</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6">
-      <c r="A25" t="s">
-        <v>497</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>1022</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" s="14" customFormat="1">
-      <c r="A26" s="14" t="s">
-        <v>865</v>
-      </c>
-      <c r="B26" s="14" t="s">
-        <v>1062</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6">
-      <c r="A27" t="s">
-        <v>654</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>1057</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>1058</v>
-      </c>
-      <c r="E27" t="s">
-        <v>1064</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6">
-      <c r="A28" t="s">
-        <v>345</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>1023</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>1058</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" s="15" customFormat="1">
-      <c r="A29" s="15" t="s">
-        <v>101</v>
-      </c>
-      <c r="B29" s="15" t="s">
-        <v>1056</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" s="14" customFormat="1">
-      <c r="A30" s="14" t="s">
-        <v>525</v>
-      </c>
-      <c r="B30" s="14" t="s">
-        <v>1051</v>
-      </c>
-    </row>
-  </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A1048467">
-    <sortCondition ref="A1:A1048467"/>
-  </sortState>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6C22C05-6386-4B49-853E-B77F21E46829}">
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="52.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="52.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="99.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" t="s">
         <v>6</v>
       </c>
       <c r="B1" t="s">
@@ -16603,617 +15842,384 @@
       <c r="C1" t="s">
         <v>19</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" s="2" customFormat="1">
+      <c r="E1" s="1" t="s">
+        <v>1013</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>1011</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="2" customFormat="1">
       <c r="A2" s="2" t="s">
-        <v>601</v>
+        <v>244</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>602</v>
+        <v>245</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>601</v>
+        <v>244</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>607</v>
+        <v>250</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>1032</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" s="2" customFormat="1">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="2" customFormat="1">
       <c r="A3" s="2" t="s">
-        <v>788</v>
+        <v>253</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>789</v>
+        <v>254</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>788</v>
+        <v>253</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>607</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>1028</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" s="2" customFormat="1">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="2" customFormat="1">
       <c r="A4" s="2" t="s">
-        <v>796</v>
+        <v>259</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>797</v>
+        <v>260</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>796</v>
+        <v>259</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>607</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>1028</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="4" customFormat="1">
-      <c r="A5" s="4" t="s">
-        <v>801</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>802</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>801</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>607</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>1030</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" s="2" customFormat="1">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="2" customFormat="1">
+      <c r="A5" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="2" customFormat="1">
       <c r="A6" s="2" t="s">
-        <v>808</v>
+        <v>268</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>809</v>
+        <v>269</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>808</v>
+        <v>268</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>607</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>1029</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" s="2" customFormat="1">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="2" customFormat="1">
       <c r="A7" s="2" t="s">
-        <v>833</v>
+        <v>272</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>834</v>
+        <v>273</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>833</v>
+        <v>272</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>607</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>1031</v>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="2" customFormat="1">
+      <c r="A8" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="2" customFormat="1" ht="16" thickBot="1">
+      <c r="A9" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="2" customFormat="1" ht="16" thickBot="1">
+      <c r="A10" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>1010</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="2" customFormat="1">
+      <c r="A11" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="4" customFormat="1">
+      <c r="A12" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="2" customFormat="1">
+      <c r="A13" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="2" customFormat="1">
+      <c r="A14" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>749</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" s="2" customFormat="1">
+      <c r="A15" s="2" t="s">
+        <v>870</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>871</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>870</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" s="2" customFormat="1">
+      <c r="A16" s="2" t="s">
+        <v>895</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>896</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>895</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" s="2" customFormat="1">
+      <c r="A17" s="2" t="s">
+        <v>903</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>904</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>903</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" s="4" customFormat="1">
+      <c r="A18" s="4" t="s">
+        <v>907</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>908</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>907</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" s="4" customFormat="1">
+      <c r="A19" s="4" t="s">
+        <v>911</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>912</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>911</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" s="2" customFormat="1">
+      <c r="A20" s="2" t="s">
+        <v>937</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>938</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>937</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" s="2" customFormat="1">
+      <c r="A21" s="2" t="s">
+        <v>946</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>947</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>946</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" s="2" customFormat="1">
+      <c r="A22" s="2" t="s">
+        <v>951</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>952</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>951</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" s="2" customFormat="1">
+      <c r="A23" s="2" t="s">
+        <v>958</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>959</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>958</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" s="2" customFormat="1">
+      <c r="A24" s="2" t="s">
+        <v>964</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>965</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>964</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" s="2" customFormat="1">
+      <c r="A25" s="2" t="s">
+        <v>981</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>982</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>981</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>250</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F2D37CA-29C3-BD49-9326-06CF486A4EFB}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
-  <cols>
-    <col min="5" max="5" width="57.83203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" s="4" customFormat="1">
-      <c r="A1" s="4" t="s">
-        <v>417</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>418</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>417</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>422</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>1048</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>1049</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" s="8" customFormat="1">
-      <c r="A2" s="8" t="s">
-        <v>574</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>575</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>574</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>422</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B4857D5-237B-E945-A0DB-32FAF0CE7CD3}">
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
-  <cols>
-    <col min="4" max="4" width="18.33203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" s="8" customFormat="1">
-      <c r="A2" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" s="8" customFormat="1">
-      <c r="A3" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" s="8" customFormat="1">
-      <c r="A4" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="2" t="s">
-        <v>584</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>585</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>584</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="2" t="s">
-        <v>593</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>594</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>593</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="2" t="s">
-        <v>360</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>361</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>360</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="2" t="s">
-        <v>360</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>367</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>360</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="2" t="s">
-        <v>360</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>371</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>360</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>365</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA47AA37-095C-2D41-ADC5-D8C2D0281F2E}">
-  <dimension ref="A1:A3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" s="1" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
-      <c r="A2" s="1" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
-      <c r="A3" s="1" t="s">
-        <v>433</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C270AD3-01ED-274B-829E-C282786A8465}">
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="35.5" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1">
-      <c r="A1" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>1026</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>1023</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" s="3" customFormat="1">
-      <c r="A2" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>206</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7511E3A-EAFE-814F-AE01-B1ED38B5D125}">
-  <dimension ref="A1:E15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="44.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="43.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.83203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" s="3" customFormat="1">
-      <c r="A2" s="3" t="s">
-        <v>387</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>388</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>387</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" s="2" customFormat="1">
-      <c r="A3" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>409</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>393</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>1019</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" s="2" customFormat="1">
-      <c r="A4" s="2" t="s">
-        <v>628</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>629</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>634</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="2" customFormat="1">
-      <c r="A5" s="2" t="s">
-        <v>638</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>639</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>642</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" s="2" customFormat="1">
-      <c r="A6" s="2" t="s">
-        <v>695</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>696</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>695</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" s="2" customFormat="1">
-      <c r="A7" s="2" t="s">
-        <v>705</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>706</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>705</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" s="2" customFormat="1">
-      <c r="A8" s="2" t="s">
-        <v>705</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>714</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>705</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" s="2" customFormat="1">
-      <c r="A9" s="2" t="s">
-        <v>705</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>719</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>705</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" s="2" customFormat="1">
-      <c r="A10" s="2" t="s">
-        <v>705</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>722</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>705</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" s="2" customFormat="1">
-      <c r="A11" s="2" t="s">
-        <v>734</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>735</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>734</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" s="2" customFormat="1">
-      <c r="A12" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>741</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" s="2" customFormat="1">
-      <c r="A13" s="2" t="s">
-        <v>705</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>841</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>705</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" s="2" customFormat="1">
-      <c r="A14" s="2" t="s">
-        <v>695</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>890</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>695</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" s="2" customFormat="1">
-      <c r="A15" s="2" t="s">
-        <v>734</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>998</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>734</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>393</v>
-      </c>
-    </row>
-  </sheetData>
+  <autoFilter ref="A1:A1048461" xr:uid="{190D282D-A498-5040-B7ED-BB0A4708E39A}"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>